<commit_message>
fix: update evaluation grid spreadsheet with latest data
</commit_message>
<xml_diff>
--- a/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
+++ b/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
@@ -266,25 +266,25 @@
     <t>-      Un outil de recueil du consentement de l’utilisateur vis-à-vis des cookies est proposé pour implémentation, ses caractéristiques techniques sont détaillées,</t>
   </si>
   <si>
-    <t>Abordé. Bannière de consentement implémentée (frontend/components/common/cookie-banner.tsx, montée dans app/layout.tsx). Caractéristiques techniques et politique documentées dans Politique_Confidentialite_CGU.md.</t>
+    <t>Non abordé. Ce critère s'évalue sur le livrable E9, un cas professionnel écrit HORS projet fil rouge : audit RGPD technique d'un site web marchand existant fourni par le certificateur. Ce cas n'est pas commencé et son sujet n'a pas été réclamé. Attendu : proposer un outil de recueil du consentement aux cookies POUR LE SITE AUDITÉ et en détailler les caractéristiques techniques. La bannière implémentée dans TaskForce prouve la capacité à le faire, elle ne se substitue pas au livrable.</t>
   </si>
   <si>
     <t>-      Une vue « politique de confidentialité et traitement des données à caractère personnel » est prévue.</t>
   </si>
   <si>
-    <t>Abordé. Vue « politique de confidentialité » présente dans l'application (frontend/app/privacy-policy/page.tsx) et sur la landing, cohérence code contre politique vérifiée.</t>
+    <t>Non abordé. Ce critère s'évalue sur le livrable E9, un cas professionnel écrit HORS projet fil rouge : audit RGPD technique d'un site web marchand existant fourni par le certificateur. Ce cas n'est pas commencé et son sujet n'a pas été réclamé. Attendu : prévoir une vue « politique de confidentialité et traitement des données à caractère personnel » pour le site audité.</t>
   </si>
   <si>
     <t>-      Un formulaire de demande d’accès aux données personnelles et le traitement correspondant est proposé pour implémentation.</t>
   </si>
   <si>
-    <t>Abordé. Droits des personnes exposés par l'API : GET /api/gdpr/export (portabilité, export JSON) et DELETE /api/gdpr/account (droit à l'effacement, anonymisation locale plus suppression de l'identité Keycloak).</t>
+    <t>Non abordé. Ce critère s'évalue sur le livrable E9, un cas professionnel écrit HORS projet fil rouge : audit RGPD technique d'un site web marchand existant fourni par le certificateur. Ce cas n'est pas commencé et son sujet n'a pas été réclamé. Attendu : proposer pour implémentation un formulaire de demande d'accès aux données personnelles et le traitement correspondant, pour le site audité.</t>
   </si>
   <si>
     <t>-      La modification des traitements collectant des données personnelles est proposée pour mettre en place un processus de double opt-in.</t>
   </si>
   <si>
-    <t>Abordé. Double opt-in implémenté et vérifié dans le code le 22/07 : la validation du code OTP marque l'adresse comme vérifiée, et la connexion est BLOQUÉE tant qu'elle ne l'est pas.</t>
+    <t>Non abordé. Ce critère s'évalue sur le livrable E9, un cas professionnel écrit HORS projet fil rouge : audit RGPD technique d'un site web marchand existant fourni par le certificateur. Ce cas n'est pas commencé et son sujet n'a pas été réclamé. Attendu : proposer la modification des traitements collectant des données personnelles afin d'y mettre en place un double opt-in, pour le site audité.</t>
   </si>
   <si>
     <t>C12. Proposer des solutions alternatives et/ou innovantes, issues de son activité de veille métier, afin de contribuer à l’atteinte de la promesse de valeur, ainsi qu’à la résolution de problèmes, lors d’un projet d’application (web, hybride, mobile ou desktop).</t>
@@ -972,7 +972,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1110,6 +1110,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2144,11 +2150,11 @@
       <c r="B39" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="C39" s="45"/>
+      <c r="C39" s="50" t="s">
+        <v>83</v>
+      </c>
       <c r="D39" s="35"/>
-      <c r="E39" s="30" t="s">
-        <v>83</v>
-      </c>
+      <c r="E39" s="23"/>
       <c r="F39" s="5"/>
     </row>
     <row r="40" ht="42.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2156,11 +2162,11 @@
       <c r="B40" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="C40" s="42"/>
+      <c r="C40" s="51" t="s">
+        <v>85</v>
+      </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="30" t="s">
-        <v>85</v>
-      </c>
+      <c r="E40" s="23"/>
       <c r="F40" s="5"/>
     </row>
     <row r="41" ht="71.25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2168,11 +2174,11 @@
       <c r="B41" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="42"/>
+      <c r="C41" s="51" t="s">
+        <v>87</v>
+      </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="30" t="s">
-        <v>87</v>
-      </c>
+      <c r="E41" s="23"/>
       <c r="F41" s="5"/>
     </row>
     <row r="42" ht="28.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2180,11 +2186,11 @@
       <c r="B42" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="42"/>
+      <c r="C42" s="51" t="s">
+        <v>89</v>
+      </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="30" t="s">
-        <v>89</v>
-      </c>
+      <c r="E42" s="23"/>
       <c r="F42" s="5"/>
     </row>
     <row r="43" ht="28.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2214,28 +2220,28 @@
       <c r="F44" s="5"/>
     </row>
     <row r="45" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C45" s="50"/>
-      <c r="D45" s="50"/>
-      <c r="E45" s="50"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="52"/>
+      <c r="E45" s="52"/>
     </row>
     <row r="46" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C46" s="50"/>
-      <c r="D46" s="50"/>
-      <c r="E46" s="50"/>
+      <c r="C46" s="52"/>
+      <c r="D46" s="52"/>
+      <c r="E46" s="52"/>
     </row>
     <row r="47" ht="15" customHeight="1" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C47" s="50"/>
-      <c r="D47" s="50"/>
-      <c r="E47" s="50"/>
+      <c r="C47" s="52"/>
+      <c r="D47" s="52"/>
+      <c r="E47" s="52"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="51" t="s">
+      <c r="A48" s="53" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="52"/>
-      <c r="C48" s="53"/>
-      <c r="D48" s="53"/>
-      <c r="E48" s="53"/>
+      <c r="B48" s="54"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
     </row>
     <row r="49" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
@@ -2293,13 +2299,13 @@
         <v>102</v>
       </c>
       <c r="C53" s="23"/>
-      <c r="D53" s="54" t="s">
+      <c r="D53" s="56" t="s">
         <v>103</v>
       </c>
       <c r="E53" s="23"/>
     </row>
     <row r="54" ht="42.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="55" t="s">
+      <c r="A54" s="57" t="s">
         <v>104</v>
       </c>
       <c r="B54" s="28" t="s">
@@ -2379,7 +2385,7 @@
       <c r="D60" s="46" t="s">
         <v>120</v>
       </c>
-      <c r="E60" s="56"/>
+      <c r="E60" s="58"/>
     </row>
     <row r="61" ht="22.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="36"/>
@@ -2409,7 +2415,7 @@
         <v>125</v>
       </c>
       <c r="C63" s="23"/>
-      <c r="D63" s="54" t="s">
+      <c r="D63" s="56" t="s">
         <v>126</v>
       </c>
       <c r="E63" s="23"/>
@@ -2571,10 +2577,10 @@
       <c r="E77" s="20"/>
     </row>
     <row r="78" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="57" t="s">
+      <c r="A78" s="59" t="s">
         <v>156</v>
       </c>
-      <c r="B78" s="58" t="s">
+      <c r="B78" s="60" t="s">
         <v>157</v>
       </c>
       <c r="C78" s="45"/>
@@ -2585,7 +2591,7 @@
     </row>
     <row r="79" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="36"/>
-      <c r="B79" s="58" t="s">
+      <c r="B79" s="60" t="s">
         <v>159</v>
       </c>
       <c r="C79" s="43" t="s">
@@ -2596,7 +2602,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="36"/>
-      <c r="B80" s="58" t="s">
+      <c r="B80" s="60" t="s">
         <v>161</v>
       </c>
       <c r="C80" s="43" t="s">
@@ -2607,7 +2613,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="25"/>
-      <c r="B81" s="58" t="s">
+      <c r="B81" s="60" t="s">
         <v>163</v>
       </c>
       <c r="C81" s="42"/>
@@ -2619,22 +2625,22 @@
     <row r="82" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
-      <c r="C82" s="59"/>
-      <c r="D82" s="59"/>
-      <c r="E82" s="59"/>
+      <c r="C82" s="61"/>
+      <c r="D82" s="61"/>
+      <c r="E82" s="61"/>
     </row>
     <row r="83" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="60"/>
-      <c r="B83" s="60"/>
-      <c r="C83" s="61"/>
-      <c r="D83" s="61"/>
-      <c r="E83" s="61"/>
+      <c r="A83" s="62"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="63"/>
+      <c r="D83" s="63"/>
+      <c r="E83" s="63"/>
     </row>
     <row r="84" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="B84" s="62"/>
+      <c r="B84" s="64"/>
       <c r="C84" s="12"/>
       <c r="D84" s="12"/>
       <c r="E84" s="12"/>
@@ -2669,7 +2675,7 @@
       <c r="A87" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="B87" s="63" t="s">
+      <c r="B87" s="65" t="s">
         <v>168</v>
       </c>
       <c r="C87" s="23"/>
@@ -2860,7 +2866,7 @@
         <v>200</v>
       </c>
       <c r="C104" s="23"/>
-      <c r="D104" s="54" t="s">
+      <c r="D104" s="56" t="s">
         <v>201</v>
       </c>
       <c r="E104" s="23"/>
@@ -2900,7 +2906,7 @@
     </row>
     <row r="108" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="25"/>
-      <c r="B108" s="64"/>
+      <c r="B108" s="66"/>
       <c r="C108" s="23"/>
       <c r="D108" s="23"/>
       <c r="E108" s="23"/>
@@ -2916,7 +2922,7 @@
       <c r="D109" s="46" t="s">
         <v>209</v>
       </c>
-      <c r="E109" s="56"/>
+      <c r="E109" s="58"/>
     </row>
     <row r="110" ht="23.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="36"/>
@@ -2924,10 +2930,10 @@
         <v>210</v>
       </c>
       <c r="C110" s="23"/>
-      <c r="D110" s="54" t="s">
+      <c r="D110" s="56" t="s">
         <v>211</v>
       </c>
-      <c r="E110" s="65"/>
+      <c r="E110" s="67"/>
     </row>
     <row r="111" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="36"/>

</xml_diff>

<commit_message>
fix: update evaluation grid with latest data
</commit_message>
<xml_diff>
--- a/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
+++ b/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
@@ -497,13 +497,13 @@
     <t>-      - Le choix des outils de mesure d’audience et de performance marketing est pertinent : les outils sont les plus performants possibles au regard du besoin et des moyens du client.</t>
   </si>
   <si>
-    <t>Non abordé. Aucun outil de mesure d'audience n'est intégré (ni Plausible, ni Matomo, ni équivalent). L'observabilité technique existe (OpenTelemetry vers SigNoz, 9 règles d'alerte) mais elle mesure la santé du service, pas l'audience marketing. Les deux ne doivent pas être confondus devant le jury.</t>
+    <t>Abordé. Outil retenu : Umami, auto-hébergé (`docker-compose.dev.yml` et `.prod.yml`). Le choix est motivé par la conformité et non par le confort : aucun cookie déposé, donc aucun consentement à recueillir, et aucun transfert hors UE, donc aucun destinataire étranger au registre des traitements. Une solution hébergée outre-Atlantique aurait contredit le retrait du fournisseur d'IA américain du 16/07 et l'auto-hébergement du modèle de langage. Mesures collectées : pages consultées, provenance, appareil, navigateur.</t>
   </si>
   <si>
     <t>-      L’intégration des outils de mesure de performance marketing est fonctionnelle.</t>
   </si>
   <si>
-    <t>Non abordé. Aucun outil de mesure de performance marketing n'est intégré, donc son intégration ne peut être qualifiée de fonctionnelle. Voir le critère précédent.</t>
+    <t>Abordé. Intégration vérifiée de bout en bout le 23/07/2026 : le service répond, sert son script de mesure, et un événement de page émis vers l'API a été retrouvé en base avec sa provenance, son navigateur et son type d'appareil. Le script est injecté sur les 16 pages via un composant unique (`AudienceTracking.astro`), et n'est émis que si les variables d'environnement sont renseignées, afin que les constructions locales et les audits Lighthouse ne polluent pas les statistiques.</t>
   </si>
   <si>
     <t>-      L’application est conforme à au moins 70% des critères d’optimisation technique SEO en vigueur.</t>
@@ -2594,22 +2594,22 @@
       <c r="B79" s="60" t="s">
         <v>159</v>
       </c>
-      <c r="C79" s="43" t="s">
+      <c r="C79" s="23"/>
+      <c r="D79" s="29"/>
+      <c r="E79" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="D79" s="29"/>
-      <c r="E79" s="23"/>
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="36"/>
       <c r="B80" s="60" t="s">
         <v>161</v>
       </c>
-      <c r="C80" s="43" t="s">
+      <c r="C80" s="23"/>
+      <c r="D80" s="29"/>
+      <c r="E80" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="D80" s="29"/>
-      <c r="E80" s="23"/>
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="25"/>

</xml_diff>

<commit_message>
docs(mémoire): met à jour la grille d'évaluation remplie
</commit_message>
<xml_diff>
--- a/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
+++ b/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
@@ -2368,10 +2368,12 @@
         <v>119</v>
       </c>
       <c r="C60" s="23"/>
-      <c r="D60" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="E60" s="55"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abordé. Le code satisfait aux revues par analyse statique : TypeScript strict sans « any », ESLint à 0 erreur sur l'ensemble du dépôt, et l'analyse statique de Semgrep et de CodeQL exécutée en intégration continue. S'y ajoutent les en-têtes de sécurité, une CSP durcie, les CORS configurés et des dépendances auditées. L'application est désormais déployée en production derrière un tunnel Cloudflare, qui assure le certificat TLS.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="36"/>
@@ -2905,10 +2907,12 @@
         <v>147</v>
       </c>
       <c r="C109" s="23"/>
-      <c r="D109" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="E109" s="55"/>
+      <c r="D109" s="23"/>
+      <c r="E109" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abordé. Processus d'industrialisation fonctionnel : l'intégration continue back (backend-tests.yml) exécute les tests avec une porte de couverture JaCoCo bloquante (mvn verify déclenchant jacoco-check) et publie le rapport, puis construit une image Docker multi-étapes publiée sur GHCR. La sécurité est automatisée par des workflows dédiés : CodeQL et Semgrep en analyse statique, Trivy pour les dépendances et la configuration, et OWASP ZAP en analyse dynamique.</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="23.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="36"/>
@@ -2916,10 +2920,12 @@
         <v>210</v>
       </c>
       <c r="C110" s="23"/>
-      <c r="D110" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="E110" s="64"/>
+      <c r="D110" s="23"/>
+      <c r="E110" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abordé. Outils de qualité cohérents et automatisés : ESLint et TypeScript strict, tests JUnit avec porte de couverture JaCoCo, et la chaîne de sécurité CodeQL, Semgrep, Trivy et OWASP ZAP, tous câblés dans des workflows GitHub Actions exécutés à chaque poussée.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="36"/>

</xml_diff>